<commit_message>
Fix SEO update wiping meta descriptions; record 2026-10-01 fixes
The 2026-09-25 apply sent each new SEO title without the existing meta
description, and Shopify cleared the description on all 33 shelves that
had one. apply now always sends the live description with the title, and
restore keeps it too (covered by a mocked regression check).

Applied on the live store 2026-10-01 and verified by read-back:
- restored the 33 meta descriptions from snapshot.json
- corrected the 26 1/2" half shelves' meta descriptions (said 28 1/2")
- corrected sizes in 3 descriptions (Spectrum 13x26x3/4, Advancer
  13x26 and 14x28)
- CoreLite octagon: titled 15" x 16", filter value 15" Diameter

changes-2026-10-01.json keeps the exact before/after values. The plan,
overrides and README are updated to match, and the README's Experro
steps now use the app's real menu names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dPTwhEiv4fMVTB38djktK
</commit_message>
<xml_diff>
--- a/kiln-shelves/plan.xlsx
+++ b/kiln-shelves/plan.xlsx
@@ -984,7 +984,7 @@
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Thickness not in title; set to Advancer standard 5/16" - confirm.</t>
+          <t>Thickness not in the old title; Advancer lists its multi-sided shelves at 5/16".</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1062,7 +1062,7 @@
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Thickness not in title; set to Advancer standard 5/16" - confirm. Vendor part no. (AKS-ADV2020F10S-1) duplicates the 20" full shelf's.</t>
+          <t>Thickness not in the old title; Advancer lists its multi-sided shelves at 5/16". Vendor part no. (AKS-ADV2020F10S-1) duplicates the 20" full shelf's.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       <c r="I9" s="3" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Thickness not in title; set to Advancer standard 5/16" - confirm.</t>
+          <t>Thickness not in the old title; Advancer lists its multi-sided shelves at 5/16".</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1218,7 +1218,7 @@
       <c r="I10" s="3" t="inlineStr"/>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Thickness not in title; set to Advancer standard 5/16" - confirm.</t>
+          <t>Thickness not in the old title; Advancer lists its multi-sided shelves at 5/16".</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1296,7 +1296,7 @@
       <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Thickness not in title; set to Advancer standard 5/16" - confirm.</t>
+          <t>Thickness not in the old title; Advancer lists its multi-sided shelves at 5/16".</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1709,156 +1709,148 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Advancer Kiln Shelf 13 x26 x 5/16" Nitride Bonded Silicon Carbide Rectangle</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Advancer Silicon Carbide Kiln Shelf - 13" x 26" Rectangle, 5/16" Thick</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>13" x 26"</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Rectangle</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>5/16"</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Advancer Kiln Shelves | Sheffield Pottery | Nitride Bonded Silicon Carbide</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Advancer Kiln Shelf 13" x 26" x 5/16" Rectangle | Sheffield Pottery</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>Description opens with "12 x28"; fix the description.</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Advancer</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>SSFADV1326</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>advancer-kiln-shelf-13-x26-x-5-16-silicon-carbide-ssfadv1326</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>gid://shopify/Product/8316337586498</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>https://www.sheffield-pottery.com/products/advancer-kiln-shelf-13-x26-x-5-16-silicon-carbide-ssfadv1326</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Advancer Kiln Shelf 14 x 28 x 5/16" Nitride Bonded Silicon Carbide Rectangle</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Advancer Silicon Carbide Kiln Shelf - 14" x 28" Rectangle, 5/16" Thick</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>14" x 28"</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Rectangle</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>5/16"</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Advancer Kiln Shelves | Sheffield Pottery | Nitride Bonded Silicon Carbide</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Advancer Kiln Shelf 14" x 28" x 5/16" Rectangle | Sheffield Pottery</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Description opens with "11 x 22"; fix the description.</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Advancer</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>SSFADV1428</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>advancer-kiln-shelf-14-x28-x-5-16-silicon-carbide-ssfadv1428</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>gid://shopify/Product/8316337848642</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>https://www.sheffield-pottery.com/products/advancer-kiln-shelf-14-x28-x-5-16-silicon-carbide-ssfadv1428</t>
         </is>
@@ -2797,12 +2789,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Cedar Heights CoreLite Semi-Hollow Kiln Shelf - 16" x 15" Full 8-Sided, 5/8" Thick</t>
+          <t>Cedar Heights CoreLite Semi-Hollow Kiln Shelf - 15" x 16" Full 8-Sided, 5/8" Thick</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>16" Diameter</t>
+          <t>15" Diameter</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2822,7 +2814,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>CoreLite Semi-Hollow Kiln Shelf 16" x 15" x 5/8" Full 8-Sided</t>
+          <t>CoreLite Semi-Hollow Kiln Shelf 15" x 16" x 5/8" Full 8-Sided</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2832,7 +2824,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Octagon listed as 16" x 15" (corner-to-corner x flat-to-flat?); filed under 16" Diameter - confirm.</t>
+          <t>Old title said 16" x 15"; sold as a 15" octagon, so filed under 15" Diameter.</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -4777,156 +4769,148 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>26 1/2" X 1" Half Round High Alumina Kiln Shelf</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Spectrum High Alumina Kiln Shelf - 26 1/2" Half Round, 1" Thick</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>26 1/2" Diameter</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>Half Round</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>1"</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>27 1/2" x 3/4" HALF ROUND HIGH ALUMINA KILN SHELF</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>Spectrum High Alumina Kiln Shelf 26 1/2" x 1" Half Round</t>
         </is>
       </c>
-      <c r="I57" s="3" t="inlineStr"/>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>Old SEO title said 27 1/2" and meta description says 28 1/2"; fix the meta description too.</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr"/>
+      <c r="J57" s="5" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>Spectrum Kiln Shelves</t>
         </is>
       </c>
-      <c r="M57" s="2" t="inlineStr">
+      <c r="M57" s="4" t="inlineStr">
         <is>
           <t>SPHA261</t>
         </is>
       </c>
-      <c r="N57" s="2" t="inlineStr">
+      <c r="N57" s="4" t="inlineStr">
         <is>
           <t>26-1-2-x-1-half-round-high-alumina-kiln-shelf</t>
         </is>
       </c>
-      <c r="O57" s="2" t="inlineStr">
+      <c r="O57" s="4" t="inlineStr">
         <is>
           <t>gid://shopify/Product/15042839904627</t>
         </is>
       </c>
-      <c r="P57" s="2" t="inlineStr">
+      <c r="P57" s="4" t="inlineStr">
         <is>
           <t>https://www.sheffield-pottery.com/products/26-1-2-x-1-half-round-high-alumina-kiln-shelf</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>26 1/2" X 3/4" Half Round High Alumina Kiln Shelf</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Spectrum High Alumina Kiln Shelf - 26 1/2" Half Round, 3/4" Thick</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>26 1/2" Diameter</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>Half Round</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr">
         <is>
           <t>3/4"</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>27 1/2" x 3/4" HALF ROUND HIGH ALUMINA KILN SHELF</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>Spectrum High Alumina Kiln Shelf 26 1/2" x 3/4" Half Round</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr"/>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>Old SEO title said 27 1/2" and meta description says 28 1/2"; fix the meta description too.</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr">
+      <c r="I58" s="5" t="inlineStr"/>
+      <c r="J58" s="5" t="inlineStr"/>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
         <is>
           <t>Spectrum Kiln Shelves</t>
         </is>
       </c>
-      <c r="M58" s="2" t="inlineStr">
+      <c r="M58" s="4" t="inlineStr">
         <is>
           <t>SPHA01</t>
         </is>
       </c>
-      <c r="N58" s="2" t="inlineStr">
+      <c r="N58" s="4" t="inlineStr">
         <is>
           <t>kiln-shelf-spha01</t>
         </is>
       </c>
-      <c r="O58" s="2" t="inlineStr">
+      <c r="O58" s="4" t="inlineStr">
         <is>
           <t>gid://shopify/Product/8316330737986</t>
         </is>
       </c>
-      <c r="P58" s="2" t="inlineStr">
+      <c r="P58" s="4" t="inlineStr">
         <is>
           <t>https://www.sheffield-pottery.com/products/kiln-shelf-spha01</t>
         </is>
@@ -5307,78 +5291,74 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>26" X 13" X 3/4" Rectangle High Alumina Kiln Shelf</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Spectrum High Alumina Kiln Shelf - 13" x 26" Rectangle, 3/4" Thick</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
         <is>
           <t>13" x 26"</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
         <is>
           <t>Rectangle</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>3/4"</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>26" x 13" x 3/4" RECTANGLE HIGH ALUMI</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>Spectrum High Alumina Kiln Shelf 13" x 26" x 3/4" Rectangle</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr"/>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>Description says 26" x 13" x 1"; title and SKU say 3/4" (the 1" version is archived). Fix the description.</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="I64" s="5" t="inlineStr"/>
+      <c r="J64" s="5" t="inlineStr"/>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="L64" s="4" t="inlineStr">
         <is>
           <t>Spectrum Kiln Shelves</t>
         </is>
       </c>
-      <c r="M64" s="2" t="inlineStr">
+      <c r="M64" s="4" t="inlineStr">
         <is>
           <t>SPHA09</t>
         </is>
       </c>
-      <c r="N64" s="2" t="inlineStr">
+      <c r="N64" s="4" t="inlineStr">
         <is>
           <t>kiln-shelf-spha09</t>
         </is>
       </c>
-      <c r="O64" s="2" t="inlineStr">
+      <c r="O64" s="4" t="inlineStr">
         <is>
           <t>gid://shopify/Product/8316331786562</t>
         </is>
       </c>
-      <c r="P64" s="2" t="inlineStr">
+      <c r="P64" s="4" t="inlineStr">
         <is>
           <t>https://www.sheffield-pottery.com/products/kiln-shelf-spha09</t>
         </is>

</xml_diff>